<commit_message>
feat(excel-prep): derive DASH viewer and editor from range
Co-Authored-By: Claude Opus 5.5 (1M context)
</commit_message>
<xml_diff>
--- a/tests/test_input/plain_small.xlsx
+++ b/tests/test_input/plain_small.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -639,6 +639,35 @@
       <c r="G6" t="inlineStr">
         <is>
           <t>0..1</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Catalog description</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>dct:description</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>rdfs:Literal</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>0..n</t>
         </is>
       </c>
     </row>

</xml_diff>